<commit_message>
Updated by บาส at 2026-08-25 03:08:22
</commit_message>
<xml_diff>
--- a/รายการแผนคอม 71.xlsx
+++ b/รายการแผนคอม 71.xlsx
@@ -1077,16 +1077,16 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
         <v>31500</v>
       </c>
       <c r="H22" t="n">
-        <v>63000</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="23">
@@ -6710,7 +6710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6857,6 +6857,68 @@
       </c>
       <c r="P2" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-25 03:08:22</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ชวก.(ก1)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์ สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I3" t="n">
+        <v>63000</v>
+      </c>
+      <c r="J3" t="n">
+        <v>31500</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-31500</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>บาส</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0002900</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ฝคท</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated by aaa at 2026-08-25 03:16:46
</commit_message>
<xml_diff>
--- a/รายการแผนคอม 71.xlsx
+++ b/รายการแผนคอม 71.xlsx
@@ -1077,16 +1077,16 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" t="n">
         <v>31500</v>
       </c>
       <c r="H22" t="n">
-        <v>31500</v>
+        <v>63000</v>
       </c>
     </row>
     <row r="23">
@@ -6710,7 +6710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6840,15 +6840,11 @@
           <t>บาส</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>0002900</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M2" t="n">
+        <v>2900</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -6902,15 +6898,11 @@
           <t>บาส</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0002900</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M3" t="n">
+        <v>2900</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -6918,6 +6910,68 @@
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-25 03:16:46</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ชวก.(ก1)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์ สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I4" t="n">
+        <v>31500</v>
+      </c>
+      <c r="J4" t="n">
+        <v>63000</v>
+      </c>
+      <c r="K4" t="n">
+        <v>31500</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated by 1 at 2026-08-25 03:18:37
</commit_message>
<xml_diff>
--- a/รายการแผนคอม 71.xlsx
+++ b/รายการแผนคอม 71.xlsx
@@ -1077,16 +1077,16 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
         <v>31500</v>
       </c>
       <c r="H22" t="n">
-        <v>63000</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="23">
@@ -6710,7 +6710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6956,22 +6956,80 @@
           <t>aaa</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>00</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>00</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>00</t>
-        </is>
-      </c>
       <c r="P4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-25 03:18:37</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ชวก.(ก1)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์ สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I5" t="n">
+        <v>63000</v>
+      </c>
+      <c r="J5" t="n">
+        <v>31500</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-31500</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated/Confirmed by 1 at 2026-08-25 07:54:24
</commit_message>
<xml_diff>
--- a/รายการแผนคอม 71.xlsx
+++ b/รายการแผนคอม 71.xlsx
@@ -477,16 +477,16 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>31500</v>
       </c>
       <c r="H2" t="n">
-        <v>94500</v>
+        <v>63000</v>
       </c>
     </row>
     <row r="3">
@@ -6710,7 +6710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6794,6 +6794,11 @@
           <t>หน่วยงานรายการ</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6852,6 +6857,7 @@
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6910,6 +6916,7 @@
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6968,6 +6975,7 @@
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7014,22 +7022,145 @@
           <t>1</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-25 07:54:24</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ฝตล.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์ สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>63000</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>ยืนยัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-25 07:54:24</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>70</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ฝตล.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์โน้ตบุ๊ก สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>94500</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>ยืนยัน</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated/Confirmed by 1 at 2026-08-25 07:54:30
</commit_message>
<xml_diff>
--- a/รายการแผนคอม 71.xlsx
+++ b/รายการแผนคอม 71.xlsx
@@ -6710,7 +6710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7162,6 +7162,132 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25 07:54:30</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ฝตล.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์ สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>63000</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>ยืนยัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25 07:54:30</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>70</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ฝตล.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์โน้ตบุ๊ก สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>94500</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>ยืนยัน</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated/Confirmed by 1 at 2026-08-25 07:55:43
</commit_message>
<xml_diff>
--- a/รายการแผนคอม 71.xlsx
+++ b/รายการแผนคอม 71.xlsx
@@ -477,16 +477,16 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
         <v>31500</v>
       </c>
       <c r="H2" t="n">
-        <v>63000</v>
+        <v>94500</v>
       </c>
     </row>
     <row r="3">
@@ -6710,7 +6710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7288,6 +7288,132 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-25 07:55:43</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ฝตล.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์ สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>94500</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-25 07:55:43</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>70</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ฝตล.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์โน้ตบุ๊ก สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>94500</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>ยืนยัน</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated/Confirmed by Test at 2026-08-27 01:55:09
</commit_message>
<xml_diff>
--- a/รายการแผนคอม 71.xlsx
+++ b/รายการแผนคอม 71.xlsx
@@ -1077,16 +1077,16 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
         <v>31500</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="23">
@@ -6710,7 +6710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6863,6 +6863,69 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-27 01:55:09</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ชวก.(ก1)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>เครื่องคอมพิวเตอร์ สำหรับงานประมวลผล พร้อมระบบปฏิบัติการ Windows</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>31500</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>31500</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test </t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>